<commit_message>
feat: add hospital and speciality matching logic and improve responsive mobile navigation and table layouts
</commit_message>
<xml_diff>
--- a/UGANDA/May/UGANDA EXPENSES MAY-2026.xlsx
+++ b/UGANDA/May/UGANDA EXPENSES MAY-2026.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25225"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\sale  and weekly report\Uganda\may for razy\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\pc\dashboards\uganda-sales-dashboard\UGANDA\May\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4867C15E-D1F9-48B4-943B-4F7014ADF211}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{C841ED64-0A19-43A3-8BCB-B78608E9BF7F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="MONEY REVEIVED" sheetId="1" r:id="rId1"/>
@@ -25,20 +24,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="183">
   <si>
     <t>Type</t>
   </si>
@@ -550,36 +541,9 @@
     <t>Campaign</t>
   </si>
   <si>
-    <t>No outcome in may and june as they all are for exam leave, so expecting outcome in july</t>
-  </si>
-  <si>
     <t>Job Kuteesa</t>
   </si>
   <si>
-    <t>4000 EURO In May 26</t>
-  </si>
-  <si>
-    <t>500 euro in may</t>
-  </si>
-  <si>
-    <t>150 euro in May 26</t>
-  </si>
-  <si>
-    <t>200 Euro in May 26</t>
-  </si>
-  <si>
-    <t>500 euro reglar but not in may due to out of stock COQ10</t>
-  </si>
-  <si>
-    <t>300 euro in may 26</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1200 Euro in may </t>
-  </si>
-  <si>
-    <t>900 Euro in May</t>
-  </si>
-  <si>
     <t>Dr Ntambi</t>
   </si>
   <si>
@@ -614,24 +578,14 @@
   </si>
   <si>
     <t>Dr Nabajjala Norah</t>
-  </si>
-  <si>
-    <t>300 Euro in May</t>
-  </si>
-  <si>
-    <t>50 Euro in May and will increase in July</t>
-  </si>
-  <si>
-    <t>400 euro</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_-[$$-409]* #,##0.00_ ;_-[$$-409]* \-#,##0.00\ ;_-[$$-409]* &quot;-&quot;??_ ;_-@_ "/>
-    <numFmt numFmtId="165" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
     <numFmt numFmtId="166" formatCode="[$UGX]\ #,##0.00"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
@@ -797,7 +751,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -888,12 +842,6 @@
     <xf numFmtId="0" fontId="7" fillId="5" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -901,10 +849,22 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{D3BA12A3-1733-4C9B-98DD-E83B53BE653D}"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1215,7 +1175,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA43902A-521A-4299-958E-E657235A615E}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1227,14 +1187,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="32" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
     </row>
     <row r="2" spans="1:12" ht="24" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1335,7 +1295,7 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="A3:A6" xr:uid="{2CF78379-FFDE-4A4E-A6F1-2629E19A2F89}">
+    <dataValidation type="list" sqref="A3:A6">
       <formula1>"OPENING BALANCE,RECEIVED,SPENT,BALANCE"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1344,7 +1304,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1730B2B1-5FBB-41E6-AB43-4F476DB0EF21}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L68"/>
   <sheetFormatPr defaultRowHeight="32.25" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1361,19 +1321,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="36" t="s">
+      <c r="A1" s="34" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="36"/>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="34"/>
+      <c r="H1" s="34"/>
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
     </row>
     <row r="2" spans="1:12" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
@@ -1436,9 +1396,7 @@
       <c r="I3" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J3" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J3" s="37"/>
       <c r="K3" s="12">
         <v>0</v>
       </c>
@@ -1470,9 +1428,7 @@
       <c r="I4" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J4" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J4" s="37"/>
       <c r="K4" s="12">
         <v>0</v>
       </c>
@@ -1504,9 +1460,7 @@
       <c r="I5" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J5" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J5" s="37"/>
       <c r="K5" s="12">
         <v>0</v>
       </c>
@@ -1538,8 +1492,8 @@
       <c r="I6" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="J6" s="8" t="s">
-        <v>175</v>
+      <c r="J6" s="35">
+        <v>200</v>
       </c>
       <c r="K6" s="12">
         <v>1</v>
@@ -1572,8 +1526,8 @@
       <c r="I7" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="J7" s="8" t="s">
-        <v>175</v>
+      <c r="J7" s="35">
+        <v>200</v>
       </c>
       <c r="K7" s="12">
         <v>2</v>
@@ -1606,8 +1560,8 @@
       <c r="I8" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="J8" s="8" t="s">
-        <v>175</v>
+      <c r="J8" s="35">
+        <v>200</v>
       </c>
       <c r="K8" s="12">
         <v>1</v>
@@ -1640,8 +1594,8 @@
       <c r="I9" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="J9" s="8" t="s">
-        <v>175</v>
+      <c r="J9" s="35">
+        <v>200</v>
       </c>
       <c r="K9" s="12">
         <v>4</v>
@@ -1674,8 +1628,8 @@
       <c r="I10" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="J10" s="8" t="s">
-        <v>175</v>
+      <c r="J10" s="35">
+        <v>200</v>
       </c>
       <c r="K10" s="12">
         <v>1</v>
@@ -1708,8 +1662,8 @@
       <c r="I11" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="J11" s="8" t="s">
-        <v>175</v>
+      <c r="J11" s="35">
+        <v>200</v>
       </c>
       <c r="K11" s="12">
         <v>2</v>
@@ -1742,8 +1696,8 @@
       <c r="I12" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="J12" s="8" t="s">
-        <v>175</v>
+      <c r="J12" s="35">
+        <v>200</v>
       </c>
       <c r="K12" s="12">
         <v>2</v>
@@ -1776,8 +1730,8 @@
       <c r="I13" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="J13" s="8" t="s">
-        <v>175</v>
+      <c r="J13" s="35">
+        <v>200</v>
       </c>
       <c r="K13" s="12">
         <v>0</v>
@@ -1810,8 +1764,8 @@
       <c r="I14" s="8" t="s">
         <v>145</v>
       </c>
-      <c r="J14" s="8" t="s">
-        <v>175</v>
+      <c r="J14" s="35">
+        <v>200</v>
       </c>
       <c r="K14" s="12">
         <v>1</v>
@@ -1844,8 +1798,8 @@
       <c r="I15" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="J15" s="8" t="s">
-        <v>175</v>
+      <c r="J15" s="35">
+        <v>200</v>
       </c>
       <c r="K15" s="12">
         <v>3</v>
@@ -1878,8 +1832,8 @@
       <c r="I16" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J16" s="8" t="s">
-        <v>194</v>
+      <c r="J16" s="35">
+        <v>400</v>
       </c>
       <c r="K16" s="12">
         <v>2</v>
@@ -1912,9 +1866,7 @@
       <c r="I17" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J17" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J17" s="37"/>
       <c r="K17" s="12">
         <v>3</v>
       </c>
@@ -1946,8 +1898,8 @@
       <c r="I18" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="J18" s="8" t="s">
-        <v>172</v>
+      <c r="J18" s="35">
+        <v>400</v>
       </c>
       <c r="K18" s="12">
         <v>2</v>
@@ -1980,9 +1932,7 @@
       <c r="I19" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J19" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J19" s="37"/>
       <c r="K19" s="12">
         <v>2</v>
       </c>
@@ -2014,8 +1964,8 @@
       <c r="I20" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="J20" s="8" t="s">
-        <v>173</v>
+      <c r="J20" s="35">
+        <v>500</v>
       </c>
       <c r="K20" s="15">
         <v>2</v>
@@ -2048,7 +1998,7 @@
       <c r="I21" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="J21" s="8">
+      <c r="J21" s="35">
         <v>1500</v>
       </c>
       <c r="K21" s="12">
@@ -2082,9 +2032,7 @@
       <c r="I22" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J22" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J22" s="37"/>
       <c r="K22" s="12">
         <v>0</v>
       </c>
@@ -2116,9 +2064,7 @@
       <c r="I23" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J23" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J23" s="37"/>
       <c r="K23" s="12">
         <v>0</v>
       </c>
@@ -2150,9 +2096,7 @@
       <c r="I24" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J24" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J24" s="37"/>
       <c r="K24" s="8">
         <v>2</v>
       </c>
@@ -2184,9 +2128,7 @@
       <c r="I25" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J25" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J25" s="37"/>
       <c r="K25" s="12">
         <v>0</v>
       </c>
@@ -2218,9 +2160,7 @@
       <c r="I26" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J26" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J26" s="37"/>
       <c r="K26" s="8">
         <v>1</v>
       </c>
@@ -2252,9 +2192,7 @@
       <c r="I27" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J27" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J27" s="37"/>
       <c r="K27" s="8">
         <v>2</v>
       </c>
@@ -2286,8 +2224,8 @@
       <c r="I28" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="J28" s="33" t="s">
-        <v>173</v>
+      <c r="J28" s="38">
+        <v>500</v>
       </c>
       <c r="K28" s="8">
         <v>2</v>
@@ -2320,9 +2258,7 @@
       <c r="I29" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J29" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J29" s="37"/>
       <c r="K29" s="12">
         <v>0</v>
       </c>
@@ -2354,8 +2290,8 @@
       <c r="I30" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="J30" s="33" t="s">
-        <v>174</v>
+      <c r="J30" s="38">
+        <v>1500</v>
       </c>
       <c r="K30" s="12">
         <v>0</v>
@@ -2388,8 +2324,8 @@
       <c r="I31" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="J31" s="33" t="s">
-        <v>175</v>
+      <c r="J31" s="38">
+        <v>200</v>
       </c>
       <c r="K31" s="8">
         <v>2</v>
@@ -2422,9 +2358,7 @@
       <c r="I32" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J32" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J32" s="37"/>
       <c r="K32" s="12">
         <v>0</v>
       </c>
@@ -2456,9 +2390,7 @@
       <c r="I33" s="22" t="s">
         <v>57</v>
       </c>
-      <c r="J33" s="22" t="s">
-        <v>176</v>
-      </c>
+      <c r="J33" s="36"/>
       <c r="K33" s="8">
         <v>1</v>
       </c>
@@ -2490,8 +2422,8 @@
       <c r="I34" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="J34" s="22" t="s">
-        <v>177</v>
+      <c r="J34" s="36">
+        <v>300</v>
       </c>
       <c r="K34" s="8">
         <v>2</v>
@@ -2524,8 +2456,8 @@
       <c r="I35" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J35" s="22" t="s">
-        <v>173</v>
+      <c r="J35" s="36">
+        <v>500</v>
       </c>
       <c r="K35" s="8">
         <v>2</v>
@@ -2558,8 +2490,8 @@
       <c r="I36" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="J36" s="22" t="s">
-        <v>177</v>
+      <c r="J36" s="36">
+        <v>300</v>
       </c>
       <c r="K36" s="8">
         <v>2</v>
@@ -2592,9 +2524,7 @@
       <c r="I37" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J37" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J37" s="37"/>
       <c r="K37" s="12">
         <v>0</v>
       </c>
@@ -2626,8 +2556,8 @@
       <c r="I38" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="J38" s="22" t="s">
-        <v>174</v>
+      <c r="J38" s="36">
+        <v>1500</v>
       </c>
       <c r="K38" s="8">
         <v>4</v>
@@ -2660,9 +2590,7 @@
       <c r="I39" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J39" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J39" s="37"/>
       <c r="K39" s="12">
         <v>0</v>
       </c>
@@ -2694,9 +2622,7 @@
       <c r="I40" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J40" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J40" s="37"/>
       <c r="K40" s="12">
         <v>0</v>
       </c>
@@ -2728,9 +2654,7 @@
       <c r="I41" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J41" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J41" s="37"/>
       <c r="K41" s="12">
         <v>0</v>
       </c>
@@ -2762,9 +2686,7 @@
       <c r="I42" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J42" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J42" s="37"/>
       <c r="K42" s="8">
         <v>2</v>
       </c>
@@ -2796,8 +2718,8 @@
       <c r="I43" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J43" s="22" t="s">
-        <v>178</v>
+      <c r="J43" s="36">
+        <v>1200</v>
       </c>
       <c r="K43" s="8">
         <v>1</v>
@@ -2830,9 +2752,7 @@
       <c r="I44" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J44" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J44" s="37"/>
       <c r="K44" s="12">
         <v>0</v>
       </c>
@@ -2864,9 +2784,7 @@
       <c r="I45" s="22" t="s">
         <v>56</v>
       </c>
-      <c r="J45" s="32" t="s">
-        <v>170</v>
-      </c>
+      <c r="J45" s="37"/>
       <c r="K45" s="8">
         <v>6</v>
       </c>
@@ -2898,7 +2816,7 @@
       <c r="I46" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="J46" s="8"/>
+      <c r="J46" s="35"/>
       <c r="K46" s="12">
         <v>0</v>
       </c>
@@ -2928,7 +2846,7 @@
       <c r="I47" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="J47" s="8"/>
+      <c r="J47" s="35"/>
       <c r="K47" s="12">
         <v>0</v>
       </c>
@@ -2957,7 +2875,7 @@
       <c r="I48" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="J48" s="8"/>
+      <c r="J48" s="35"/>
       <c r="K48" s="12">
         <v>0</v>
       </c>
@@ -2986,8 +2904,8 @@
       <c r="I49" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="J49" s="8" t="s">
-        <v>193</v>
+      <c r="J49" s="35">
+        <v>50</v>
       </c>
       <c r="K49" s="8">
         <v>3</v>
@@ -3017,7 +2935,7 @@
       <c r="I50" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="J50" s="8"/>
+      <c r="J50" s="35"/>
       <c r="K50" s="12">
         <v>0</v>
       </c>
@@ -3046,8 +2964,8 @@
       <c r="I51" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="J51" s="8" t="s">
-        <v>193</v>
+      <c r="J51" s="35">
+        <v>50</v>
       </c>
       <c r="K51" s="8">
         <v>3</v>
@@ -3077,7 +2995,7 @@
       <c r="I52" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="J52" s="8"/>
+      <c r="J52" s="35"/>
       <c r="K52" s="12">
         <v>0</v>
       </c>
@@ -3106,7 +3024,7 @@
       <c r="I53" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="J53" s="8"/>
+      <c r="J53" s="35"/>
       <c r="K53" s="12">
         <v>0</v>
       </c>
@@ -3135,7 +3053,7 @@
       <c r="I54" s="22" t="s">
         <v>144</v>
       </c>
-      <c r="J54" s="8"/>
+      <c r="J54" s="35"/>
       <c r="K54" s="12">
         <v>0</v>
       </c>
@@ -3143,7 +3061,7 @@
     <row r="55" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="6"/>
       <c r="B55" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C55" s="8" t="s">
         <v>32</v>
@@ -3164,8 +3082,8 @@
       <c r="I55" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="J55" s="8" t="s">
-        <v>192</v>
+      <c r="J55" s="35">
+        <v>300</v>
       </c>
       <c r="K55" s="12">
         <v>1</v>
@@ -3174,7 +3092,7 @@
     <row r="56" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="6"/>
       <c r="B56" s="8" t="s">
-        <v>180</v>
+        <v>171</v>
       </c>
       <c r="C56" s="8" t="s">
         <v>32</v>
@@ -3195,7 +3113,7 @@
       <c r="I56" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="J56" s="8"/>
+      <c r="J56" s="35"/>
       <c r="K56" s="12">
         <v>0</v>
       </c>
@@ -3203,7 +3121,7 @@
     <row r="57" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="6"/>
       <c r="B57" s="8" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
       <c r="C57" s="8" t="s">
         <v>32</v>
@@ -3224,7 +3142,7 @@
       <c r="I57" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="J57" s="8"/>
+      <c r="J57" s="35"/>
       <c r="K57" s="12">
         <v>0</v>
       </c>
@@ -3232,7 +3150,7 @@
     <row r="58" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="6"/>
       <c r="B58" s="8" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="C58" s="8" t="s">
         <v>32</v>
@@ -3253,7 +3171,7 @@
       <c r="I58" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="J58" s="8"/>
+      <c r="J58" s="35"/>
       <c r="K58" s="12">
         <v>0</v>
       </c>
@@ -3261,7 +3179,7 @@
     <row r="59" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="6"/>
       <c r="B59" s="8" t="s">
-        <v>183</v>
+        <v>174</v>
       </c>
       <c r="C59" s="8" t="s">
         <v>32</v>
@@ -3282,7 +3200,7 @@
       <c r="I59" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="J59" s="8"/>
+      <c r="J59" s="35"/>
       <c r="K59" s="12">
         <v>0</v>
       </c>
@@ -3290,7 +3208,7 @@
     <row r="60" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="6"/>
       <c r="B60" s="8" t="s">
-        <v>184</v>
+        <v>175</v>
       </c>
       <c r="C60" s="8" t="s">
         <v>32</v>
@@ -3311,7 +3229,7 @@
       <c r="I60" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="J60" s="8"/>
+      <c r="J60" s="35"/>
       <c r="K60" s="12">
         <v>0</v>
       </c>
@@ -3319,7 +3237,7 @@
     <row r="61" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="6"/>
       <c r="B61" s="8" t="s">
-        <v>185</v>
+        <v>176</v>
       </c>
       <c r="C61" s="8" t="s">
         <v>32</v>
@@ -3340,7 +3258,7 @@
       <c r="I61" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="J61" s="8"/>
+      <c r="J61" s="35"/>
       <c r="K61" s="12">
         <v>0</v>
       </c>
@@ -3348,7 +3266,7 @@
     <row r="62" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="6"/>
       <c r="B62" s="8" t="s">
-        <v>186</v>
+        <v>177</v>
       </c>
       <c r="C62" s="8" t="s">
         <v>32</v>
@@ -3369,8 +3287,8 @@
       <c r="I62" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="J62" s="8" t="s">
-        <v>192</v>
+      <c r="J62" s="35">
+        <v>300</v>
       </c>
       <c r="K62" s="12">
         <v>2</v>
@@ -3379,7 +3297,7 @@
     <row r="63" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="6"/>
       <c r="B63" s="8" t="s">
-        <v>187</v>
+        <v>178</v>
       </c>
       <c r="C63" s="8" t="s">
         <v>32</v>
@@ -3400,7 +3318,7 @@
       <c r="I63" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="J63" s="8"/>
+      <c r="J63" s="35"/>
       <c r="K63" s="12">
         <v>0</v>
       </c>
@@ -3408,7 +3326,7 @@
     <row r="64" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="6"/>
       <c r="B64" s="8" t="s">
-        <v>188</v>
+        <v>179</v>
       </c>
       <c r="C64" s="8" t="s">
         <v>32</v>
@@ -3429,7 +3347,7 @@
       <c r="I64" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="J64" s="8"/>
+      <c r="J64" s="35"/>
       <c r="K64" s="12">
         <v>0</v>
       </c>
@@ -3437,7 +3355,7 @@
     <row r="65" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="6"/>
       <c r="B65" s="8" t="s">
-        <v>189</v>
+        <v>180</v>
       </c>
       <c r="C65" s="8" t="s">
         <v>32</v>
@@ -3458,8 +3376,8 @@
       <c r="I65" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="J65" s="8" t="s">
-        <v>192</v>
+      <c r="J65" s="35">
+        <v>300</v>
       </c>
       <c r="K65" s="12">
         <v>1</v>
@@ -3468,7 +3386,7 @@
     <row r="66" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="6"/>
       <c r="B66" s="8" t="s">
-        <v>190</v>
+        <v>181</v>
       </c>
       <c r="C66" s="8" t="s">
         <v>32</v>
@@ -3489,7 +3407,7 @@
       <c r="I66" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="J66" s="8"/>
+      <c r="J66" s="35"/>
       <c r="K66" s="12">
         <v>0</v>
       </c>
@@ -3497,7 +3415,7 @@
     <row r="67" spans="1:11" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="6"/>
       <c r="B67" s="8" t="s">
-        <v>191</v>
+        <v>182</v>
       </c>
       <c r="C67" s="8" t="s">
         <v>32</v>
@@ -3518,7 +3436,7 @@
       <c r="I67" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="J67" s="8"/>
+      <c r="J67" s="35"/>
       <c r="K67" s="12">
         <v>0</v>
       </c>
@@ -3547,8 +3465,8 @@
       <c r="I68" s="22" t="s">
         <v>145</v>
       </c>
-      <c r="J68" s="8" t="s">
-        <v>179</v>
+      <c r="J68" s="35">
+        <v>900</v>
       </c>
       <c r="K68" s="12">
         <v>0</v>
@@ -3563,7 +3481,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93E2FE39-060A-403B-8F06-1975D4D26EF4}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:G8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3573,15 +3491,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="32" t="s">
         <v>106</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
-      <c r="F1" s="35"/>
-      <c r="G1" s="35"/>
+      <c r="B1" s="33"/>
+      <c r="C1" s="33"/>
+      <c r="D1" s="33"/>
+      <c r="E1" s="33"/>
+      <c r="F1" s="33"/>
+      <c r="G1" s="33"/>
     </row>
     <row r="2" spans="1:7" ht="24" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">

</xml_diff>